<commit_message>
replace md with subset version + rerun
</commit_message>
<xml_diff>
--- a/data/04_manual_tabular/Seddaiu2016.xlsx
+++ b/data/04_manual_tabular/Seddaiu2016.xlsx
@@ -1570,10 +1570,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:I324"/>
+  <dimension ref="A1:I363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="16.711"/>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="22.711"/>
     <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="21.711"/>
     <col min="3" max="3" bestFit="1" customWidth="1" hidden="false" width="18.711"/>
     <col min="4" max="4" bestFit="1" customWidth="1" hidden="false" width="19.711"/>
@@ -16807,6 +16807,1839 @@
       <c r="I324" t="inlineStr">
         <is>
           <t>about one month after sowing applied in number of days from the first of January at 126 (98-169)</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2002_maize</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2002_maize</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2002_maize</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2003_maize</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2003_maize</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2003_maize</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2004_maize</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2004_maize</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2004_maize</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2005_maize</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2005_maize</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2005_maize</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2006_maize</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2006_maize</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2006_maize</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2007_maize</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2007_maize</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2007_maize</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2008_maize</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2008_maize</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2008_maize</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2009_maize</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2009_maize</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2009_maize</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2010_maize</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2010_maize</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2010_maize</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2011_maize</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2011_maize</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2011_maize</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2012_maize</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2012_maize</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2012_maize</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2013_maize</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2013_maize</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2013_maize</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2014_maize</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>N0_maize</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2014_maize</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>N1_maize</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Seddaiu2016_2014_maize</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>N2_maize</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>